<commit_message>
Group supplementary results under data and add supported rice windows
Move eight saved result files into data/supplementary without changing their contents. Add data indexes and a verified 16,875-row export that excludes empty empirical windows. Update scripts, provenance, README and table source paths while preserving the original six Excel files.
</commit_message>
<xml_diff>
--- a/tables/Supplementary_Tables.xlsx
+++ b/tables/Supplementary_Tables.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="1" r:id="Rd2564eb6dc144b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="2" r:id="Re2d26ad941f54fa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="3" r:id="R026240136a354ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="4" r:id="Re44404f010f64269"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5A" sheetId="5" r:id="R4553fadfeedb4ac5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5B" sheetId="6" r:id="R35b9aac8c43c4c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="1" r:id="R1b1cebdeecf74ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="2" r:id="R4d25ddb08a3b4441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="3" r:id="R65ea023693c74ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="4" r:id="R9d77c2e2ab1c4b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5A" sheetId="5" r:id="R08d6a221a68244f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5B" sheetId="6" r:id="R1b81967e6bea4b91"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -679,7 +679,7 @@
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="27" t="str">
-        <x:v>Source: results/descriptive/Supplementary_Data_S1_threshold_sim.tsv</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S1_threshold_sim.tsv</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
       <x:c r="C18" s="2"/>
@@ -968,7 +968,7 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="27" t="str">
-        <x:v>Source: results/descriptive/Supplementary_Data_S2_peakshift_sim.tsv</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S2_peakshift_sim.tsv</x:v>
       </x:c>
       <x:c r="B14" s="2"/>
       <x:c r="C14" s="2"/>
@@ -1376,7 +1376,7 @@
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="27" t="str">
-        <x:v>Source: results/f2/benchmark_protocol.json</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S5/benchmark_protocol.json</x:v>
       </x:c>
       <x:c r="B22" s="2"/>
       <x:c r="C22" s="2"/>
@@ -1699,7 +1699,7 @@
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="27" t="str">
-        <x:v>Source: results/f2/benchmark_verified_summary.tsv</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S5/benchmark_verified_summary.tsv</x:v>
       </x:c>
       <x:c r="B17" s="2"/>
       <x:c r="C17" s="2"/>
@@ -2106,7 +2106,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="27" t="str">
-        <x:v>Source: results/empirical/empirical_summary.tsv and six original Excel files in data/.</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S6/empirical_summary.tsv and six original Excel files in data/.</x:v>
       </x:c>
       <x:c r="B24" s="2"/>
       <x:c r="C24" s="2"/>
@@ -2665,7 +2665,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="27" t="str">
-        <x:v>Source: results/empirical/empirical_summary.tsv; coordinates in the manuscript captions.</x:v>
+        <x:v>Source: data/supplementary/Supplementary_Data_S6/empirical_summary.tsv; coordinates in the manuscript captions.</x:v>
       </x:c>
       <x:c r="B24" s="2"/>
       <x:c r="C24" s="2"/>

</xml_diff>